<commit_message>
src/ creation + setup.py method created
</commit_message>
<xml_diff>
--- a/notes/LIBELLULA journal.xlsx
+++ b/notes/LIBELLULA journal.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0037e56ddff3a368/Desktop/Libellula/notes/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Miguel\OneDrive\Desktop\Libellula\notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{1ABF8704-F42D-4ADD-B462-98794C3F457C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DCAE8843-0306-4583-AB2B-71E159B6B122}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ACF7916-EFB3-44C1-82C7-E4E40F0748CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{CC99F97F-3E72-4FEA-AA64-B39819E65309}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="40">
   <si>
     <t>PLANEJAMENTO LIBELLULA (secreto)</t>
   </si>
@@ -170,6 +170,18 @@
   </si>
   <si>
     <t>Indeterminado-indeterminado</t>
+  </si>
+  <si>
+    <t>Quarta-feira, 25/02/26</t>
+  </si>
+  <si>
+    <t>23h00-01h30</t>
+  </si>
+  <si>
+    <t>Sem trabalho executado</t>
+  </si>
+  <si>
+    <t>1) Separação entre notebooks com o método 'setup()' e com o modelo EPF. Antes estavam no mesmo notebook. Agora viraram dois diferentes.                                                              2) Criei um 'setup.py' na pasta 'src/' para permitir a importação ilimitada do método para todos os notebooks. O 'setup.py' está em 'src/'.</t>
   </si>
 </sst>
 </file>
@@ -667,7 +679,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6A98371-216A-4D1C-8D7B-786B21A1BFEF}">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="150" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="12.7109375" style="10" customWidth="1"/>
@@ -824,8 +836,21 @@
       <c r="B8" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="C8" s="23"/>
-      <c r="E8" s="12"/>
+      <c r="C8" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="G8" s="19" t="s">
+        <v>20</v>
+      </c>
       <c r="H8" s="24" t="s">
         <v>33</v>
       </c>
@@ -840,11 +865,44 @@
       <c r="C9" s="23" t="s">
         <v>31</v>
       </c>
+      <c r="D9" s="17" t="s">
+        <v>18</v>
+      </c>
       <c r="E9" s="12" t="s">
         <v>32</v>
+      </c>
+      <c r="F9" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="G9" s="19" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="150" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="G10" s="19" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>